<commit_message>
is someone actually reading this or may I the only one
</commit_message>
<xml_diff>
--- a/sample_data_generator/sample_data/sample.xlsx
+++ b/sample_data_generator/sample_data/sample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\omnissiah\Project\nodejs\react\Smart_Data_Management\sample_data_generator\sample_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{781FCD56-ED9A-4709-8E48-54BDEC2B27DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{973E8D79-C463-4F2C-AD41-3FDAE6C9C320}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -554,7 +554,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -593,9 +593,6 @@
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2348,7 +2345,7 @@
       <c r="AT1" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="AU1" s="15" t="s">
+      <c r="AU1" s="1" t="s">
         <v>155</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added report like view
</commit_message>
<xml_diff>
--- a/sample_data_generator/sample_data/sample.xlsx
+++ b/sample_data_generator/sample_data/sample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\omnissiah\Project\nodejs\react\Smart_Data_Management\sample_data_generator\sample_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67EB8F82-AF0D-47B0-8DA5-3B8A2AD3371C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA42EF4F-2F7D-45BE-9FC6-8E3853748973}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -971,7 +971,7 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>

</xml_diff>